<commit_message>
Close held lanes: OW live deck, economics_url, PR #95 Caribbean
- Publish Ocean Whisperer Google Sheet + wire economics_url on partner JSON
- Build live Slides deck (Curaçao composited bg, hospitality ladder, 255 ops)
- PR #95: consolidate caribbean-mobility → caribbean; ABC routes in abc-islands market
- Add publish_partner_economics.py + apply_caribbean_consolidation.py
</commit_message>
<xml_diff>
--- a/finance/_refresh_caribbean.xlsx
+++ b/finance/_refresh_caribbean.xlsx
@@ -2369,19 +2369,9 @@
         <f>((D4*O4/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG4" s="31" t="n">
-        <v>27418</v>
-      </c>
-      <c r="AH4" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI4" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG4" s="31" t="n"/>
+      <c r="AH4" s="32" t="n"/>
+      <c r="AI4" s="32" t="n"/>
       <c r="AJ4" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2431,11 +2421,7 @@
           <t>MODELED dive-transfer band (Klein Bonaire). To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY4" s="44" t="inlineStr">
-        <is>
-          <t>bonaire dive transfer pool</t>
-        </is>
-      </c>
+      <c r="AY4" s="44" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
@@ -2568,19 +2554,9 @@
         <f>((D5*O5/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D5*O5*VLOOKUP(B5,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG5" s="31" t="n">
-        <v>53850</v>
-      </c>
-      <c r="AH5" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI5" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG5" s="31" t="n"/>
+      <c r="AH5" s="32" t="n"/>
+      <c r="AI5" s="32" t="n"/>
       <c r="AJ5" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2630,11 +2606,7 @@
           <t>MODELED short town/cruise→dive-resort transfer. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY5" s="44" t="inlineStr">
-        <is>
-          <t>bonaire cruise → dive-resort cluster</t>
-        </is>
-      </c>
+      <c r="AY5" s="44" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -2767,19 +2739,9 @@
         <f>((D6*O6/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D6*O6*VLOOKUP(B6,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG6" s="31" t="n">
-        <v>216000</v>
-      </c>
-      <c r="AH6" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI6" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG6" s="31" t="n"/>
+      <c r="AH6" s="32" t="n"/>
+      <c r="AI6" s="32" t="n"/>
       <c r="AJ6" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2829,11 +2791,7 @@
           <t>MODELED premium air→resort transfer band. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY6" s="44" t="inlineStr">
-        <is>
-          <t>aruba airport → resort</t>
-        </is>
-      </c>
+      <c r="AY6" s="44" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -2966,19 +2924,9 @@
         <f>((D7*O7/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D7*O7*VLOOKUP(B7,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG7" s="31" t="n">
-        <v>102000</v>
-      </c>
-      <c r="AH7" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI7" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG7" s="31" t="n"/>
+      <c r="AH7" s="32" t="n"/>
+      <c r="AI7" s="32" t="n"/>
       <c r="AJ7" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3028,11 +2976,7 @@
           <t>MODELED premium cruise-shore / resort transfer band. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY7" s="44" t="inlineStr">
-        <is>
-          <t>aruba cruise → resort strip</t>
-        </is>
-      </c>
+      <c r="AY7" s="44" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
@@ -3165,19 +3109,9 @@
         <f>((D8*O8/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG8" s="31" t="n">
-        <v>83489</v>
-      </c>
-      <c r="AH8" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI8" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG8" s="31" t="n"/>
+      <c r="AH8" s="32" t="n"/>
+      <c r="AI8" s="32" t="n"/>
       <c r="AJ8" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3227,11 +3161,7 @@
           <t>MODELED premium cruise/town→resort transfer band. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY8" s="44" t="inlineStr">
-        <is>
-          <t>curacao cruise → resort cluster</t>
-        </is>
-      </c>
+      <c r="AY8" s="44" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -3364,19 +3294,9 @@
         <f>((D9*O9/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D9*O9*VLOOKUP(B9,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG9" s="31" t="n">
-        <v>84029</v>
-      </c>
-      <c r="AH9" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI9" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG9" s="31" t="n"/>
+      <c r="AH9" s="32" t="n"/>
+      <c r="AI9" s="32" t="n"/>
       <c r="AJ9" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3426,11 +3346,7 @@
           <t>MODELED premium air→resort transfer band. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY9" s="44" t="inlineStr">
-        <is>
-          <t>curacao airport → south-coast resorts</t>
-        </is>
-      </c>
+      <c r="AY9" s="44" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -3563,19 +3479,9 @@
         <f>((D10*O10/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG10" s="31" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AH10" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI10" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG10" s="31" t="n"/>
+      <c r="AH10" s="32" t="n"/>
+      <c r="AI10" s="32" t="n"/>
       <c r="AJ10" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3625,11 +3531,7 @@
           <t>MODELED premium seasonal excursion. To be finalized in cascade with season_days.</t>
         </is>
       </c>
-      <c r="AY10" s="44" t="inlineStr">
-        <is>
-          <t>ABC broad-footprint default slice</t>
-        </is>
-      </c>
+      <c r="AY10" s="44" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -3762,19 +3664,9 @@
         <f>((D11*O11/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D11*O11*VLOOKUP(B11,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG11" s="31" t="n">
-        <v>55480</v>
-      </c>
-      <c r="AH11" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="AI11" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="AG11" s="31" t="n"/>
+      <c r="AH11" s="32" t="n"/>
+      <c r="AI11" s="32" t="n"/>
       <c r="AJ11" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3824,11 +3716,7 @@
           <t>MODELED against the live Divi Divi/EZ Air Curaçao↔Bonaire one-way fare band (~$90-130); sea transfer priced below air. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY11" s="44" t="inlineStr">
-        <is>
-          <t>inter_island_air_substitution_pool Curaçao↔Bonaire high-frequency turboprop</t>
-        </is>
-      </c>
+      <c r="AY11" s="44" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="45" t="inlineStr">

</xml_diff>